<commit_message>
Fix z-score blank: replace AGGREGATE with array formulas for avg/stdev
AGGREGATE(1/8, 6, range) was silently failing when BDH cells contain NA()
during Bloomberg's async load phase — IFERROR caught the failure and wrote
"" to the stat cells, making z-score return "" too.

Replace with array formulas {=AVERAGE(IF(ISNUMBER(range),range))} and
{=STDEV(IF(ISNUMBER(range),range))} which filter out NA() cells natively
and recalculate correctly once Bloomberg populates the BDH history.

https://claude.ai/code/session_01Nox5BUq1EsCWnyKPLiaUt6
</commit_message>
<xml_diff>
--- a/Workbook/Most.Traded.Universe.xlsx
+++ b/Workbook/Most.Traded.Universe.xlsx
@@ -44728,11 +44728,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f>IFERROR(AGGREGATE(1,6,P3:AI3),"")</f>
+        <f t="array" ref="N3">IFERROR(AVERAGE(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="O3">
-        <f>IFERROR(AGGREGATE(8,6,P3:AI3),"")</f>
+        <f t="array" ref="O3">IFERROR(STDEV(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="P3">
@@ -44866,11 +44866,11 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f>IFERROR(AGGREGATE(1,6,P4:AI4),"")</f>
+        <f t="array" ref="N4">IFERROR(AVERAGE(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="O4">
-        <f>IFERROR(AGGREGATE(8,6,P4:AI4),"")</f>
+        <f t="array" ref="O4">IFERROR(STDEV(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="P4">
@@ -45004,11 +45004,11 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <f>IFERROR(AGGREGATE(1,6,P5:AI5),"")</f>
+        <f t="array" ref="N5">IFERROR(AVERAGE(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="O5">
-        <f>IFERROR(AGGREGATE(8,6,P5:AI5),"")</f>
+        <f t="array" ref="O5">IFERROR(STDEV(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="P5">
@@ -45142,11 +45142,11 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <f>IFERROR(AGGREGATE(1,6,P6:AI6),"")</f>
+        <f t="array" ref="N6">IFERROR(AVERAGE(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="O6">
-        <f>IFERROR(AGGREGATE(8,6,P6:AI6),"")</f>
+        <f t="array" ref="O6">IFERROR(STDEV(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="P6">
@@ -45280,11 +45280,11 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <f>IFERROR(AGGREGATE(1,6,P7:AI7),"")</f>
+        <f t="array" ref="N7">IFERROR(AVERAGE(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="O7">
-        <f>IFERROR(AGGREGATE(8,6,P7:AI7),"")</f>
+        <f t="array" ref="O7">IFERROR(STDEV(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="P7">
@@ -45418,11 +45418,11 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <f>IFERROR(AGGREGATE(1,6,P8:AI8),"")</f>
+        <f t="array" ref="N8">IFERROR(AVERAGE(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="O8">
-        <f>IFERROR(AGGREGATE(8,6,P8:AI8),"")</f>
+        <f t="array" ref="O8">IFERROR(STDEV(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="P8">
@@ -45556,11 +45556,11 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <f>IFERROR(AGGREGATE(1,6,P9:AI9),"")</f>
+        <f t="array" ref="N9">IFERROR(AVERAGE(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="O9">
-        <f>IFERROR(AGGREGATE(8,6,P9:AI9),"")</f>
+        <f t="array" ref="O9">IFERROR(STDEV(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="P9">
@@ -45694,11 +45694,11 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <f>IFERROR(AGGREGATE(1,6,P10:AI10),"")</f>
+        <f t="array" ref="N10">IFERROR(AVERAGE(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="O10">
-        <f>IFERROR(AGGREGATE(8,6,P10:AI10),"")</f>
+        <f t="array" ref="O10">IFERROR(STDEV(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="P10">
@@ -45832,11 +45832,11 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <f>IFERROR(AGGREGATE(1,6,P11:AI11),"")</f>
+        <f t="array" ref="N11">IFERROR(AVERAGE(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="O11">
-        <f>IFERROR(AGGREGATE(8,6,P11:AI11),"")</f>
+        <f t="array" ref="O11">IFERROR(STDEV(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="P11">
@@ -45970,11 +45970,11 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <f>IFERROR(AGGREGATE(1,6,P12:AI12),"")</f>
+        <f t="array" ref="N12">IFERROR(AVERAGE(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="O12">
-        <f>IFERROR(AGGREGATE(8,6,P12:AI12),"")</f>
+        <f t="array" ref="O12">IFERROR(STDEV(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="P12">
@@ -55525,11 +55525,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f>IFERROR(AGGREGATE(1,6,P3:AI3),"")</f>
+        <f t="array" ref="N3">IFERROR(AVERAGE(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="O3">
-        <f>IFERROR(AGGREGATE(8,6,P3:AI3),"")</f>
+        <f t="array" ref="O3">IFERROR(STDEV(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="P3">
@@ -55663,11 +55663,11 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f>IFERROR(AGGREGATE(1,6,P4:AI4),"")</f>
+        <f t="array" ref="N4">IFERROR(AVERAGE(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="O4">
-        <f>IFERROR(AGGREGATE(8,6,P4:AI4),"")</f>
+        <f t="array" ref="O4">IFERROR(STDEV(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="P4">
@@ -55801,11 +55801,11 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <f>IFERROR(AGGREGATE(1,6,P5:AI5),"")</f>
+        <f t="array" ref="N5">IFERROR(AVERAGE(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="O5">
-        <f>IFERROR(AGGREGATE(8,6,P5:AI5),"")</f>
+        <f t="array" ref="O5">IFERROR(STDEV(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="P5">
@@ -55939,11 +55939,11 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <f>IFERROR(AGGREGATE(1,6,P6:AI6),"")</f>
+        <f t="array" ref="N6">IFERROR(AVERAGE(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="O6">
-        <f>IFERROR(AGGREGATE(8,6,P6:AI6),"")</f>
+        <f t="array" ref="O6">IFERROR(STDEV(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="P6">
@@ -56077,11 +56077,11 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <f>IFERROR(AGGREGATE(1,6,P7:AI7),"")</f>
+        <f t="array" ref="N7">IFERROR(AVERAGE(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="O7">
-        <f>IFERROR(AGGREGATE(8,6,P7:AI7),"")</f>
+        <f t="array" ref="O7">IFERROR(STDEV(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="P7">
@@ -56215,11 +56215,11 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <f>IFERROR(AGGREGATE(1,6,P8:AI8),"")</f>
+        <f t="array" ref="N8">IFERROR(AVERAGE(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="O8">
-        <f>IFERROR(AGGREGATE(8,6,P8:AI8),"")</f>
+        <f t="array" ref="O8">IFERROR(STDEV(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="P8">
@@ -56353,11 +56353,11 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <f>IFERROR(AGGREGATE(1,6,P9:AI9),"")</f>
+        <f t="array" ref="N9">IFERROR(AVERAGE(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="O9">
-        <f>IFERROR(AGGREGATE(8,6,P9:AI9),"")</f>
+        <f t="array" ref="O9">IFERROR(STDEV(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="P9">
@@ -56491,11 +56491,11 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <f>IFERROR(AGGREGATE(1,6,P10:AI10),"")</f>
+        <f t="array" ref="N10">IFERROR(AVERAGE(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="O10">
-        <f>IFERROR(AGGREGATE(8,6,P10:AI10),"")</f>
+        <f t="array" ref="O10">IFERROR(STDEV(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="P10">
@@ -56629,11 +56629,11 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <f>IFERROR(AGGREGATE(1,6,P11:AI11),"")</f>
+        <f t="array" ref="N11">IFERROR(AVERAGE(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="O11">
-        <f>IFERROR(AGGREGATE(8,6,P11:AI11),"")</f>
+        <f t="array" ref="O11">IFERROR(STDEV(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="P11">
@@ -56767,11 +56767,11 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <f>IFERROR(AGGREGATE(1,6,P12:AI12),"")</f>
+        <f t="array" ref="N12">IFERROR(AVERAGE(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="O12">
-        <f>IFERROR(AGGREGATE(8,6,P12:AI12),"")</f>
+        <f t="array" ref="O12">IFERROR(STDEV(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="P12">
@@ -64525,11 +64525,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f>IFERROR(AGGREGATE(1,6,P3:AI3),"")</f>
+        <f t="array" ref="N3">IFERROR(AVERAGE(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="O3">
-        <f>IFERROR(AGGREGATE(8,6,P3:AI3),"")</f>
+        <f t="array" ref="O3">IFERROR(STDEV(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="P3">
@@ -64663,11 +64663,11 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f>IFERROR(AGGREGATE(1,6,P4:AI4),"")</f>
+        <f t="array" ref="N4">IFERROR(AVERAGE(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="O4">
-        <f>IFERROR(AGGREGATE(8,6,P4:AI4),"")</f>
+        <f t="array" ref="O4">IFERROR(STDEV(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="P4">
@@ -64801,11 +64801,11 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <f>IFERROR(AGGREGATE(1,6,P5:AI5),"")</f>
+        <f t="array" ref="N5">IFERROR(AVERAGE(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="O5">
-        <f>IFERROR(AGGREGATE(8,6,P5:AI5),"")</f>
+        <f t="array" ref="O5">IFERROR(STDEV(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="P5">
@@ -64939,11 +64939,11 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <f>IFERROR(AGGREGATE(1,6,P6:AI6),"")</f>
+        <f t="array" ref="N6">IFERROR(AVERAGE(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="O6">
-        <f>IFERROR(AGGREGATE(8,6,P6:AI6),"")</f>
+        <f t="array" ref="O6">IFERROR(STDEV(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="P6">
@@ -65077,11 +65077,11 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <f>IFERROR(AGGREGATE(1,6,P7:AI7),"")</f>
+        <f t="array" ref="N7">IFERROR(AVERAGE(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="O7">
-        <f>IFERROR(AGGREGATE(8,6,P7:AI7),"")</f>
+        <f t="array" ref="O7">IFERROR(STDEV(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="P7">
@@ -65215,11 +65215,11 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <f>IFERROR(AGGREGATE(1,6,P8:AI8),"")</f>
+        <f t="array" ref="N8">IFERROR(AVERAGE(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="O8">
-        <f>IFERROR(AGGREGATE(8,6,P8:AI8),"")</f>
+        <f t="array" ref="O8">IFERROR(STDEV(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="P8">
@@ -65353,11 +65353,11 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <f>IFERROR(AGGREGATE(1,6,P9:AI9),"")</f>
+        <f t="array" ref="N9">IFERROR(AVERAGE(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="O9">
-        <f>IFERROR(AGGREGATE(8,6,P9:AI9),"")</f>
+        <f t="array" ref="O9">IFERROR(STDEV(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="P9">
@@ -65491,11 +65491,11 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <f>IFERROR(AGGREGATE(1,6,P10:AI10),"")</f>
+        <f t="array" ref="N10">IFERROR(AVERAGE(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="O10">
-        <f>IFERROR(AGGREGATE(8,6,P10:AI10),"")</f>
+        <f t="array" ref="O10">IFERROR(STDEV(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="P10">
@@ -65629,11 +65629,11 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <f>IFERROR(AGGREGATE(1,6,P11:AI11),"")</f>
+        <f t="array" ref="N11">IFERROR(AVERAGE(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="O11">
-        <f>IFERROR(AGGREGATE(8,6,P11:AI11),"")</f>
+        <f t="array" ref="O11">IFERROR(STDEV(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="P11">
@@ -65767,11 +65767,11 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <f>IFERROR(AGGREGATE(1,6,P12:AI12),"")</f>
+        <f t="array" ref="N12">IFERROR(AVERAGE(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="O12">
-        <f>IFERROR(AGGREGATE(8,6,P12:AI12),"")</f>
+        <f t="array" ref="O12">IFERROR(STDEV(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="P12">
@@ -72437,11 +72437,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f>IFERROR(AGGREGATE(1,6,P3:AI3),"")</f>
+        <f t="array" ref="N3">IFERROR(AVERAGE(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="O3">
-        <f>IFERROR(AGGREGATE(8,6,P3:AI3),"")</f>
+        <f t="array" ref="O3">IFERROR(STDEV(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="P3">
@@ -72575,11 +72575,11 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f>IFERROR(AGGREGATE(1,6,P4:AI4),"")</f>
+        <f t="array" ref="N4">IFERROR(AVERAGE(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="O4">
-        <f>IFERROR(AGGREGATE(8,6,P4:AI4),"")</f>
+        <f t="array" ref="O4">IFERROR(STDEV(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="P4">
@@ -72713,11 +72713,11 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <f>IFERROR(AGGREGATE(1,6,P5:AI5),"")</f>
+        <f t="array" ref="N5">IFERROR(AVERAGE(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="O5">
-        <f>IFERROR(AGGREGATE(8,6,P5:AI5),"")</f>
+        <f t="array" ref="O5">IFERROR(STDEV(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="P5">
@@ -72851,11 +72851,11 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <f>IFERROR(AGGREGATE(1,6,P6:AI6),"")</f>
+        <f t="array" ref="N6">IFERROR(AVERAGE(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="O6">
-        <f>IFERROR(AGGREGATE(8,6,P6:AI6),"")</f>
+        <f t="array" ref="O6">IFERROR(STDEV(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="P6">
@@ -72989,11 +72989,11 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <f>IFERROR(AGGREGATE(1,6,P7:AI7),"")</f>
+        <f t="array" ref="N7">IFERROR(AVERAGE(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="O7">
-        <f>IFERROR(AGGREGATE(8,6,P7:AI7),"")</f>
+        <f t="array" ref="O7">IFERROR(STDEV(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="P7">
@@ -73127,11 +73127,11 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <f>IFERROR(AGGREGATE(1,6,P8:AI8),"")</f>
+        <f t="array" ref="N8">IFERROR(AVERAGE(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="O8">
-        <f>IFERROR(AGGREGATE(8,6,P8:AI8),"")</f>
+        <f t="array" ref="O8">IFERROR(STDEV(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="P8">
@@ -73265,11 +73265,11 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <f>IFERROR(AGGREGATE(1,6,P9:AI9),"")</f>
+        <f t="array" ref="N9">IFERROR(AVERAGE(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="O9">
-        <f>IFERROR(AGGREGATE(8,6,P9:AI9),"")</f>
+        <f t="array" ref="O9">IFERROR(STDEV(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="P9">
@@ -73403,11 +73403,11 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <f>IFERROR(AGGREGATE(1,6,P10:AI10),"")</f>
+        <f t="array" ref="N10">IFERROR(AVERAGE(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="O10">
-        <f>IFERROR(AGGREGATE(8,6,P10:AI10),"")</f>
+        <f t="array" ref="O10">IFERROR(STDEV(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="P10">
@@ -73541,11 +73541,11 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <f>IFERROR(AGGREGATE(1,6,P11:AI11),"")</f>
+        <f t="array" ref="N11">IFERROR(AVERAGE(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="O11">
-        <f>IFERROR(AGGREGATE(8,6,P11:AI11),"")</f>
+        <f t="array" ref="O11">IFERROR(STDEV(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="P11">
@@ -73679,11 +73679,11 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <f>IFERROR(AGGREGATE(1,6,P12:AI12),"")</f>
+        <f t="array" ref="N12">IFERROR(AVERAGE(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="O12">
-        <f>IFERROR(AGGREGATE(8,6,P12:AI12),"")</f>
+        <f t="array" ref="O12">IFERROR(STDEV(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="P12">
@@ -79805,11 +79805,11 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f>IFERROR(AGGREGATE(1,6,P3:AI3),"")</f>
+        <f t="array" ref="N3">IFERROR(AVERAGE(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="O3">
-        <f>IFERROR(AGGREGATE(8,6,P3:AI3),"")</f>
+        <f t="array" ref="O3">IFERROR(STDEV(IF(ISNUMBER(P3:AI3),P3:AI3)),"")</f>
         <v>0</v>
       </c>
       <c r="P3">
@@ -79943,11 +79943,11 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <f>IFERROR(AGGREGATE(1,6,P4:AI4),"")</f>
+        <f t="array" ref="N4">IFERROR(AVERAGE(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="O4">
-        <f>IFERROR(AGGREGATE(8,6,P4:AI4),"")</f>
+        <f t="array" ref="O4">IFERROR(STDEV(IF(ISNUMBER(P4:AI4),P4:AI4)),"")</f>
         <v>0</v>
       </c>
       <c r="P4">
@@ -80081,11 +80081,11 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <f>IFERROR(AGGREGATE(1,6,P5:AI5),"")</f>
+        <f t="array" ref="N5">IFERROR(AVERAGE(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="O5">
-        <f>IFERROR(AGGREGATE(8,6,P5:AI5),"")</f>
+        <f t="array" ref="O5">IFERROR(STDEV(IF(ISNUMBER(P5:AI5),P5:AI5)),"")</f>
         <v>0</v>
       </c>
       <c r="P5">
@@ -80219,11 +80219,11 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <f>IFERROR(AGGREGATE(1,6,P6:AI6),"")</f>
+        <f t="array" ref="N6">IFERROR(AVERAGE(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="O6">
-        <f>IFERROR(AGGREGATE(8,6,P6:AI6),"")</f>
+        <f t="array" ref="O6">IFERROR(STDEV(IF(ISNUMBER(P6:AI6),P6:AI6)),"")</f>
         <v>0</v>
       </c>
       <c r="P6">
@@ -80357,11 +80357,11 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <f>IFERROR(AGGREGATE(1,6,P7:AI7),"")</f>
+        <f t="array" ref="N7">IFERROR(AVERAGE(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="O7">
-        <f>IFERROR(AGGREGATE(8,6,P7:AI7),"")</f>
+        <f t="array" ref="O7">IFERROR(STDEV(IF(ISNUMBER(P7:AI7),P7:AI7)),"")</f>
         <v>0</v>
       </c>
       <c r="P7">
@@ -80495,11 +80495,11 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <f>IFERROR(AGGREGATE(1,6,P8:AI8),"")</f>
+        <f t="array" ref="N8">IFERROR(AVERAGE(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="O8">
-        <f>IFERROR(AGGREGATE(8,6,P8:AI8),"")</f>
+        <f t="array" ref="O8">IFERROR(STDEV(IF(ISNUMBER(P8:AI8),P8:AI8)),"")</f>
         <v>0</v>
       </c>
       <c r="P8">
@@ -80633,11 +80633,11 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <f>IFERROR(AGGREGATE(1,6,P9:AI9),"")</f>
+        <f t="array" ref="N9">IFERROR(AVERAGE(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="O9">
-        <f>IFERROR(AGGREGATE(8,6,P9:AI9),"")</f>
+        <f t="array" ref="O9">IFERROR(STDEV(IF(ISNUMBER(P9:AI9),P9:AI9)),"")</f>
         <v>0</v>
       </c>
       <c r="P9">
@@ -80771,11 +80771,11 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <f>IFERROR(AGGREGATE(1,6,P10:AI10),"")</f>
+        <f t="array" ref="N10">IFERROR(AVERAGE(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="O10">
-        <f>IFERROR(AGGREGATE(8,6,P10:AI10),"")</f>
+        <f t="array" ref="O10">IFERROR(STDEV(IF(ISNUMBER(P10:AI10),P10:AI10)),"")</f>
         <v>0</v>
       </c>
       <c r="P10">
@@ -80909,11 +80909,11 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <f>IFERROR(AGGREGATE(1,6,P11:AI11),"")</f>
+        <f t="array" ref="N11">IFERROR(AVERAGE(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="O11">
-        <f>IFERROR(AGGREGATE(8,6,P11:AI11),"")</f>
+        <f t="array" ref="O11">IFERROR(STDEV(IF(ISNUMBER(P11:AI11),P11:AI11)),"")</f>
         <v>0</v>
       </c>
       <c r="P11">
@@ -81047,11 +81047,11 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <f>IFERROR(AGGREGATE(1,6,P12:AI12),"")</f>
+        <f t="array" ref="N12">IFERROR(AVERAGE(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="O12">
-        <f>IFERROR(AGGREGATE(8,6,P12:AI12),"")</f>
+        <f t="array" ref="O12">IFERROR(STDEV(IF(ISNUMBER(P12:AI12),P12:AI12)),"")</f>
         <v>0</v>
       </c>
       <c r="P12">

</xml_diff>